<commit_message>
updated credit model and added functionality. Made the code within the functional code oaradigm.
</commit_message>
<xml_diff>
--- a/Proyecto2/Tasa de interés.xlsx
+++ b/Proyecto2/Tasa de interés.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luism/Desktop/8-ITESO/Módelos de Crédito/Proyecto2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24CE844A-232E-9C49-9261-8814AC666854}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55D5D2D0-33B8-D04F-B43E-0D111CAA37CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{A29ECE82-7D40-644D-A928-16A1ACA67412}"/>
   </bookViews>
@@ -18,14 +18,8 @@
   <definedNames>
     <definedName name="_xlchart.v1.0" hidden="1">Hoja1!$B$3:$B$9</definedName>
     <definedName name="_xlchart.v1.1" hidden="1">Hoja1!$C$3:$C$9</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">Hoja1!$B$3:$B$9</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">Hoja1!$C$3:$C$9</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">Hoja1!$B$3:$B$9</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">Hoja1!$C$3:$C$9</definedName>
-    <definedName name="_xlchart.v2.4" hidden="1">Hoja1!$B$3:$B$9</definedName>
-    <definedName name="_xlchart.v2.5" hidden="1">Hoja1!$C$3:$C$9</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -82,6 +76,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0000%"/>
+  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -141,14 +138,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -904,8 +902,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="3780693" y="684824"/>
-              <a:ext cx="6310922" cy="3301022"/>
+              <a:off x="3772878" y="678962"/>
+              <a:ext cx="6271845" cy="3269761"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -1255,101 +1253,100 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD44646C-231B-0B44-A6E2-4704C0F68ECA}">
-  <dimension ref="B2:C13"/>
+  <dimension ref="B2:C18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="17.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="6"/>
+      <c r="C2" s="7"/>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="2">
-        <v>6.7699999999999996E-2</v>
+      <c r="C3" s="3">
+        <v>3.1699999999999999E-2</v>
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="3">
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="4">
         <f>C12*C13</f>
         <v>9.4500000000000001E-3</v>
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="2">
-        <v>5.0000000000000001E-3</v>
+      <c r="C6" s="3">
+        <v>8.8900000000000003E-3</v>
       </c>
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="2">
-        <v>5.0000000000000001E-3</v>
+      <c r="C7" s="3">
+        <v>1.7000000000000001E-2</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="5">
-        <v>5.0000000000000001E-3</v>
+        <v>1.2E-2</v>
       </c>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="4">
         <f>SUM(C3:C8)</f>
-        <v>0.12814999999999999</v>
-      </c>
-    </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
+        <v>0.11503999999999999</v>
+      </c>
     </row>
     <row r="11" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="6"/>
+      <c r="C11" s="7"/>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>3</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="1">
         <v>2.7E-2</v>
       </c>
     </row>
     <row r="13" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13" s="1">
         <v>0.35</v>
       </c>
+    </row>
+    <row r="18" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C18" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>